<commit_message>
respondemos 4 preguntas de negocio con nuestros datos, usando groupby y gráficos, realizando tambien el reto planteado punto cinco
</commit_message>
<xml_diff>
--- a/consolidado_limpio.xlsx
+++ b/consolidado_limpio.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1488,6 +1488,732 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>16/06/2026</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Camiseta basica</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>6</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Felipe Torres</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Transferencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>09/06/2026</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Camiseta basica</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>5</v>
+      </c>
+      <c r="E34" t="n">
+        <v>34000</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>18/06/2026</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Teclado mecanico</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Andres Gomez</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Transferencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>05/07/2026</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Mouse inalambrico</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="n">
+        <v>152700</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Sin Asignar</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Jean clasico</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>4</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Laura Diaz</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Medias deportivas</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>4</v>
+      </c>
+      <c r="E38" t="n">
+        <v>157700</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Andres Gomez</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>11/06/2026</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Cargador USB-C</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" t="n">
+        <v>78100</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Camila Ruiz</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Medias deportivas</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>7</v>
+      </c>
+      <c r="E40" t="n">
+        <v>78000</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Felipe Torres</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Parlante portatil</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" t="n">
+        <v>127500</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Sofia Mena</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Chaqueta impermeable</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>5</v>
+      </c>
+      <c r="E42" t="n">
+        <v>86700</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Felipe Torres</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Cargador USB-C</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>3</v>
+      </c>
+      <c r="E43" t="n">
+        <v>98800</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Camila Ruiz</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Parlante portatil</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>4</v>
+      </c>
+      <c r="E44" t="n">
+        <v>40200</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Andres Gomez</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Medias deportivas</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>8</v>
+      </c>
+      <c r="E45" t="n">
+        <v>18200</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Laura Diaz</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Jean clasico</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>4</v>
+      </c>
+      <c r="E46" t="n">
+        <v>159900</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Camila Ruiz</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Gorra deportiva</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" t="n">
+        <v>36200</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Felipe Torres</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Cargador USB-C</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>7</v>
+      </c>
+      <c r="E48" t="n">
+        <v>174100</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Sofia Mena</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Cargador USB-C</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>6</v>
+      </c>
+      <c r="E49" t="n">
+        <v>87300</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Sofia Mena</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Camiseta basica</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>4</v>
+      </c>
+      <c r="E50" t="n">
+        <v>25600</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Camila Ruiz</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Medias deportivas</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" t="n">
+        <v>26700</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Camila Ruiz</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Camiseta basica</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>6</v>
+      </c>
+      <c r="E52" t="n">
+        <v>26700</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Andres Gomez</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Gorra deportiva</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>3</v>
+      </c>
+      <c r="E53" t="n">
+        <v>134400</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Sofia Mena</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Jean clasico</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>7</v>
+      </c>
+      <c r="E54" t="n">
+        <v>46400</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Camila Ruiz</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>